<commit_message>
Després del primer dia de poda
</commit_message>
<xml_diff>
--- a/data/at/at_network/edges.xlsx
+++ b/data/at/at_network/edges.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\network\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\at\at_network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70792806-4AC9-4C81-8ED4-BEFA8C6537FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29606938-AC26-4E91-AA8D-A5A5488E107A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{306F75E9-4DFE-4518-8798-1CA0D2BB102C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="34">
   <si>
     <t>source</t>
   </si>
@@ -102,84 +102,6 @@
   </si>
   <si>
     <t>E-700</t>
-  </si>
-  <si>
-    <t>0-1</t>
-  </si>
-  <si>
-    <t>1-2</t>
-  </si>
-  <si>
-    <t>2-3</t>
-  </si>
-  <si>
-    <t>3-4</t>
-  </si>
-  <si>
-    <t>4-5</t>
-  </si>
-  <si>
-    <t>4-22</t>
-  </si>
-  <si>
-    <t>5-6</t>
-  </si>
-  <si>
-    <t>6-22</t>
-  </si>
-  <si>
-    <t>6-7</t>
-  </si>
-  <si>
-    <t>7-8</t>
-  </si>
-  <si>
-    <t>8-9</t>
-  </si>
-  <si>
-    <t>9-10</t>
-  </si>
-  <si>
-    <t>10-11</t>
-  </si>
-  <si>
-    <t>11-12</t>
-  </si>
-  <si>
-    <t>12-13</t>
-  </si>
-  <si>
-    <t>13-14</t>
-  </si>
-  <si>
-    <t>14-15</t>
-  </si>
-  <si>
-    <t>15-16</t>
-  </si>
-  <si>
-    <t>16-17</t>
-  </si>
-  <si>
-    <t>17-18</t>
-  </si>
-  <si>
-    <t>18-21</t>
-  </si>
-  <si>
-    <t>11-19</t>
-  </si>
-  <si>
-    <t>19-20</t>
-  </si>
-  <si>
-    <t>20-21</t>
-  </si>
-  <si>
-    <t>22-23</t>
-  </si>
-  <si>
-    <t>23-24</t>
   </si>
   <si>
     <t>SS-3000</t>
@@ -260,9 +182,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -627,34 +555,34 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="G1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="H1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="I1" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="J1" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="K1" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="L1" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="M1" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="N1" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="O1" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -935,8 +863,8 @@
       <c r="D7" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>21</v>
+      <c r="E7" s="2">
+        <v>0.01</v>
       </c>
       <c r="F7">
         <v>350</v>
@@ -988,8 +916,8 @@
       <c r="D8" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>22</v>
+      <c r="E8" s="2">
+        <v>1.02</v>
       </c>
       <c r="F8">
         <v>350</v>
@@ -1041,8 +969,8 @@
       <c r="D9" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>23</v>
+      <c r="E9" s="2">
+        <v>2.0299999999999998</v>
       </c>
       <c r="F9">
         <v>350</v>
@@ -1094,8 +1022,8 @@
       <c r="D10" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>24</v>
+      <c r="E10" s="3">
+        <v>3.04</v>
       </c>
       <c r="F10">
         <v>350</v>
@@ -1147,8 +1075,8 @@
       <c r="D11" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>25</v>
+      <c r="E11" s="3">
+        <v>4.05</v>
       </c>
       <c r="F11">
         <v>350</v>
@@ -1200,8 +1128,8 @@
       <c r="D12" t="s">
         <v>6</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>26</v>
+      <c r="E12" s="3">
+        <v>4.22</v>
       </c>
       <c r="F12">
         <v>80</v>
@@ -1253,8 +1181,8 @@
       <c r="D13" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>27</v>
+      <c r="E13" s="3">
+        <v>5.0599999999999996</v>
       </c>
       <c r="F13">
         <v>300</v>
@@ -1306,8 +1234,8 @@
       <c r="D14" t="s">
         <v>6</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>28</v>
+      <c r="E14" s="3">
+        <v>6.22</v>
       </c>
       <c r="F14">
         <v>100</v>
@@ -1359,8 +1287,8 @@
       <c r="D15" t="s">
         <v>6</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>29</v>
+      <c r="E15" s="3">
+        <v>6.07</v>
       </c>
       <c r="F15">
         <v>300</v>
@@ -1412,8 +1340,8 @@
       <c r="D16" t="s">
         <v>6</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>30</v>
+      <c r="E16" s="3">
+        <v>7.08</v>
       </c>
       <c r="F16">
         <v>300</v>
@@ -1465,8 +1393,8 @@
       <c r="D17" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>31</v>
+      <c r="E17" s="3">
+        <v>8.09</v>
       </c>
       <c r="F17">
         <v>300</v>
@@ -1518,8 +1446,8 @@
       <c r="D18" t="s">
         <v>6</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>32</v>
+      <c r="E18" s="3">
+        <v>9.1</v>
       </c>
       <c r="F18">
         <v>300</v>
@@ -1571,8 +1499,8 @@
       <c r="D19" t="s">
         <v>6</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>33</v>
+      <c r="E19" s="3">
+        <v>10.11</v>
       </c>
       <c r="F19">
         <v>250</v>
@@ -1624,8 +1552,8 @@
       <c r="D20" t="s">
         <v>6</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>34</v>
+      <c r="E20" s="3">
+        <v>11.12</v>
       </c>
       <c r="F20">
         <v>200</v>
@@ -1677,8 +1605,8 @@
       <c r="D21" t="s">
         <v>6</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>35</v>
+      <c r="E21" s="3">
+        <v>12.13</v>
       </c>
       <c r="F21">
         <v>200</v>
@@ -1730,8 +1658,8 @@
       <c r="D22" t="s">
         <v>6</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>36</v>
+      <c r="E22" s="3">
+        <v>13.14</v>
       </c>
       <c r="F22">
         <v>150</v>
@@ -1783,8 +1711,8 @@
       <c r="D23" t="s">
         <v>6</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>37</v>
+      <c r="E23" s="3">
+        <v>14.15</v>
       </c>
       <c r="F23">
         <v>150</v>
@@ -1836,8 +1764,8 @@
       <c r="D24" t="s">
         <v>6</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>38</v>
+      <c r="E24" s="3">
+        <v>15.16</v>
       </c>
       <c r="F24">
         <v>150</v>
@@ -1889,8 +1817,8 @@
       <c r="D25" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>39</v>
+      <c r="E25" s="3">
+        <v>16.170000000000002</v>
       </c>
       <c r="F25">
         <v>80</v>
@@ -1942,8 +1870,8 @@
       <c r="D26" t="s">
         <v>6</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>40</v>
+      <c r="E26" s="3">
+        <v>17.18</v>
       </c>
       <c r="F26">
         <v>80</v>
@@ -1995,8 +1923,8 @@
       <c r="D27" t="s">
         <v>6</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>41</v>
+      <c r="E27" s="3">
+        <v>18.21</v>
       </c>
       <c r="F27">
         <v>80</v>
@@ -2048,8 +1976,8 @@
       <c r="D28" t="s">
         <v>6</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>42</v>
+      <c r="E28" s="3">
+        <v>11.19</v>
       </c>
       <c r="F28">
         <v>250</v>
@@ -2101,8 +2029,8 @@
       <c r="D29" t="s">
         <v>6</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>43</v>
+      <c r="E29" s="3">
+        <v>19.2</v>
       </c>
       <c r="F29">
         <v>200</v>
@@ -2154,8 +2082,8 @@
       <c r="D30" t="s">
         <v>6</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>44</v>
+      <c r="E30" s="3">
+        <v>20.21</v>
       </c>
       <c r="F30">
         <v>200</v>
@@ -2207,8 +2135,8 @@
       <c r="D31" t="s">
         <v>6</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>45</v>
+      <c r="E31" s="3">
+        <v>22.23</v>
       </c>
       <c r="F31">
         <v>100</v>
@@ -2260,8 +2188,8 @@
       <c r="D32" t="s">
         <v>6</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>46</v>
+      <c r="E32" s="3">
+        <v>23.24</v>
       </c>
       <c r="F32">
         <v>100</v>
@@ -2311,7 +2239,7 @@
         <v>10</v>
       </c>
       <c r="D33" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="E33" s="1">
         <v>51000</v>
@@ -2364,7 +2292,7 @@
         <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="E34" s="1">
         <v>53000</v>
@@ -4257,7 +4185,7 @@
         <v>15</v>
       </c>
       <c r="D70" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E70" s="1">
         <v>4600.01</v>
@@ -4310,7 +4238,7 @@
         <v>15</v>
       </c>
       <c r="D71" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E71" s="1">
         <v>4671</v>
@@ -4363,7 +4291,7 @@
         <v>0</v>
       </c>
       <c r="D72" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E72" s="1">
         <v>4670</v>
@@ -4380,7 +4308,7 @@
         <v>25</v>
       </c>
       <c r="D73" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E73" s="1">
         <v>4600.0200000000004</v>
@@ -4433,7 +4361,7 @@
         <v>25</v>
       </c>
       <c r="D74" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E74" s="1">
         <v>4651</v>

</xml_diff>